<commit_message>
Tests promociones y modificadores
</commit_message>
<xml_diff>
--- a/Web/TestCases/Login.xlsx
+++ b/Web/TestCases/Login.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nerea QA\PycharmProjects\KOVAI\Web\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{80FC9867-2AF8-4AE1-A97A-A88976D6638E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16124479-D56A-43C6-A652-B6BB9822B013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="26850" windowHeight="8040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
   <si>
     <t>Num</t>
   </si>
@@ -32,9 +32,6 @@
   </si>
   <si>
     <t>Pasos</t>
-  </si>
-  <si>
-    <t>Login</t>
   </si>
   <si>
     <t>I try to login with wrong user</t>
@@ -98,13 +95,38 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1Cxs_yuyLHFT1JsmgWJW-SEwL_8VR9ryI/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>LOGIN001</t>
+  </si>
+  <si>
+    <t>LOGIN002</t>
+  </si>
+  <si>
+    <t>LOGIN003</t>
+  </si>
+  <si>
+    <t>LOGIN004</t>
+  </si>
+  <si>
+    <t>Login page home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. The user sees the Login page
+</t>
+  </si>
+  <si>
+    <t>1. The login page home is correctly.</t>
+  </si>
+  <si>
+    <t>LOGIN005</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,6 +138,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -127,6 +150,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -188,24 +217,7 @@
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6565"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -220,56 +232,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF6565"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -576,9 +538,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="41.5703125" customWidth="1"/>
     <col min="5" max="6" width="33.42578125" customWidth="1"/>
@@ -599,16 +562,16 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="H1" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -616,20 +579,20 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H2" s="1"/>
     </row>
@@ -638,86 +601,107 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>19</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F3" s="3"/>
       <c r="G3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>23</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="D4" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="2"/>
+        <v>16</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="G5" s="4" t="s">
         <v>16</v>
       </c>
       <c r="H5" s="2"/>
     </row>
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="2"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:G5">
-    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="OK">
+  <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="G2:G6">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="KO">
+      <formula>NOT(ISERROR(SEARCH("KO",G2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G5">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="KO">
-      <formula>NOT(ISERROR(SEARCH("KO",G2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="H3" r:id="rId1" xr:uid="{7414C937-D2D7-4D9C-BADD-CF4D3CE8EE08}"/>
+    <hyperlink ref="H4" r:id="rId1" xr:uid="{7414C937-D2D7-4D9C-BADD-CF4D3CE8EE08}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>